<commit_message>
(#274.2) WalkCapacity rework completed :D
</commit_message>
<xml_diff>
--- a/Assets/Resources/datasheets/EntitiesData.xlsx
+++ b/Assets/Resources/datasheets/EntitiesData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODING\UNITY\subrunner\Assets\Resources\datasheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED7B3FF-9DAF-4B1F-BBB9-E5F2D265A3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74231874-9044-4F7F-B04C-9A31C1139010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{BDB0EA0F-F215-4C7B-BC70-96EDBA517C3F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
   <si>
     <t>Agent Type</t>
   </si>
@@ -97,6 +97,21 @@
   </si>
   <si>
     <t>particles_rate</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>transp</t>
+  </si>
+  <si>
+    <t>black</t>
+  </si>
+  <si>
+    <t>purple</t>
+  </si>
+  <si>
+    <t>red</t>
   </si>
 </sst>
 </file>
@@ -1055,68 +1070,158 @@
       <c r="B5" s="11">
         <v>3</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
+      <c r="C5" s="11">
+        <v>1</v>
+      </c>
+      <c r="D5" s="11">
+        <v>1.3</v>
+      </c>
+      <c r="E5" s="11">
+        <v>3</v>
+      </c>
+      <c r="F5" s="11">
+        <v>2.9</v>
+      </c>
+      <c r="G5" s="11">
+        <v>3</v>
+      </c>
+      <c r="H5" s="11">
+        <v>3</v>
+      </c>
+      <c r="I5" s="11">
+        <v>2.8</v>
+      </c>
+      <c r="J5" s="11">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="6" spans="1:46" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
+      <c r="B6" s="11">
+        <v>4</v>
+      </c>
+      <c r="C6" s="11">
+        <v>2</v>
+      </c>
+      <c r="D6" s="11">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E6" s="11">
+        <v>4.5</v>
+      </c>
+      <c r="F6" s="11">
+        <v>5.2</v>
+      </c>
+      <c r="G6" s="11">
+        <v>6</v>
+      </c>
+      <c r="H6" s="11">
+        <v>5</v>
+      </c>
+      <c r="I6" s="11">
+        <v>3.8</v>
+      </c>
+      <c r="J6" s="11">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="7" spans="1:46" s="8" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
+      <c r="B7" s="13">
+        <v>0</v>
+      </c>
+      <c r="C7" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="D7" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="E7" s="13">
+        <v>0.1</v>
+      </c>
+      <c r="F7" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0.4</v>
+      </c>
+      <c r="H7" s="13">
+        <v>0</v>
+      </c>
+      <c r="I7" s="13">
+        <v>0</v>
+      </c>
+      <c r="J7" s="13">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:46" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
+      <c r="B8" s="1">
+        <v>30</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1">
+        <v>30</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
+        <v>30</v>
+      </c>
+      <c r="I8" s="1">
+        <v>30</v>
+      </c>
+      <c r="J8" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" spans="1:46" s="8" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="B9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="10" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>

</xml_diff>

<commit_message>
(#274.4) AttackCapacity re adapted
new OverlapHealthDetector that replace PreyDetector
new IAData that holds a SocialData with range detection +
friendly skin list
dangerous skin list
prey skin list

ClosestBeingSensor use the new HealthDetector
AttackCapacity + AttackAction updated

the "dev" skin still does not exist oopsie
sometimes the cats can't attack the zombo properly it seems ?
</commit_message>
<xml_diff>
--- a/Assets/Resources/datasheets/EntitiesData.xlsx
+++ b/Assets/Resources/datasheets/EntitiesData.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODING\UNITY\subrunner\Assets\Resources\datasheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74231874-9044-4F7F-B04C-9A31C1139010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A58AAA66-129A-4060-BDF4-160445C25F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{BDB0EA0F-F215-4C7B-BC70-96EDBA517C3F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{BDB0EA0F-F215-4C7B-BC70-96EDBA517C3F}"/>
   </bookViews>
   <sheets>
-    <sheet name="MotorData" sheetId="1" r:id="rId1"/>
-    <sheet name="WalkData" sheetId="3" r:id="rId2"/>
+    <sheet name="SocialData" sheetId="6" r:id="rId1"/>
+    <sheet name="AttackData" sheetId="5" r:id="rId2"/>
+    <sheet name="MotorData" sheetId="1" r:id="rId3"/>
+    <sheet name="WalkData" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="55">
   <si>
     <t>Agent Type</t>
   </si>
@@ -112,6 +114,96 @@
   </si>
   <si>
     <t>red</t>
+  </si>
+  <si>
+    <t>AttackData</t>
+  </si>
+  <si>
+    <t>damage</t>
+  </si>
+  <si>
+    <t>distance to attack</t>
+  </si>
+  <si>
+    <t>random damage modifier</t>
+  </si>
+  <si>
+    <t>single hit</t>
+  </si>
+  <si>
+    <t>split damage</t>
+  </si>
+  <si>
+    <t>perforant attack</t>
+  </si>
+  <si>
+    <t>attack duration</t>
+  </si>
+  <si>
+    <t>attack duration random variation</t>
+  </si>
+  <si>
+    <t>unstoppable rate</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>Cyber Rat</t>
+  </si>
+  <si>
+    <t>Excluded Tags</t>
+  </si>
+  <si>
+    <t>Robot</t>
+  </si>
+  <si>
+    <t>Cats</t>
+  </si>
+  <si>
+    <t>SocialData</t>
+  </si>
+  <si>
+    <t>range detection</t>
+  </si>
+  <si>
+    <t>friendly skins</t>
+  </si>
+  <si>
+    <t>dangerous skins</t>
+  </si>
+  <si>
+    <t>prey skins</t>
+  </si>
+  <si>
+    <t>zombo, cyber_rat, ghost, qwin</t>
+  </si>
+  <si>
+    <t>cat, perso, nobody, spider</t>
+  </si>
+  <si>
+    <t>rat, cat, perso, nobody, zombo, qwin</t>
+  </si>
+  <si>
+    <t>perso, zombo</t>
+  </si>
+  <si>
+    <t>rat, cat, perso, nobody, npc, spider, qwin, dev</t>
+  </si>
+  <si>
+    <t>zombo, rat, cyber_rat, perso, qwin, dev</t>
+  </si>
+  <si>
+    <t>zombo, nobody, perso, cat, spider, dev</t>
+  </si>
+  <si>
+    <t>zombo, rat, cyber_rat, qwin, dev</t>
+  </si>
+  <si>
+    <t>zombo, cat, dev</t>
   </si>
 </sst>
 </file>
@@ -155,7 +247,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -207,11 +299,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -245,6 +361,41 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -579,6 +730,942 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9299B342-E93E-4268-BF2B-FAA1E374A3CB}">
+  <dimension ref="A1:AU23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="33.7109375" style="3" customWidth="1"/>
+    <col min="2" max="19" width="19.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:47" s="6" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="5"/>
+      <c r="Z1" s="5"/>
+      <c r="AA1" s="5"/>
+      <c r="AB1" s="5"/>
+      <c r="AC1" s="5"/>
+      <c r="AD1" s="5"/>
+      <c r="AE1" s="5"/>
+      <c r="AF1" s="5"/>
+      <c r="AG1" s="5"/>
+      <c r="AH1" s="5"/>
+      <c r="AI1" s="5"/>
+      <c r="AJ1" s="5"/>
+      <c r="AK1" s="5"/>
+      <c r="AL1" s="5"/>
+      <c r="AM1" s="5"/>
+      <c r="AN1" s="5"/>
+      <c r="AO1" s="5"/>
+      <c r="AP1" s="5"/>
+      <c r="AQ1" s="5"/>
+      <c r="AR1" s="5"/>
+      <c r="AS1" s="5"/>
+      <c r="AT1" s="5"/>
+      <c r="AU1" s="5"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="K2" s="11"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="K3" s="11"/>
+    </row>
+    <row r="4" spans="1:47" s="8" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="K4" s="13"/>
+    </row>
+    <row r="5" spans="1:47" s="24" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23">
+        <v>15</v>
+      </c>
+      <c r="D5" s="23">
+        <v>15</v>
+      </c>
+      <c r="E5" s="23">
+        <v>15</v>
+      </c>
+      <c r="F5" s="23">
+        <v>15</v>
+      </c>
+      <c r="G5" s="23">
+        <v>15</v>
+      </c>
+      <c r="H5" s="23">
+        <v>15</v>
+      </c>
+      <c r="I5" s="23">
+        <v>15</v>
+      </c>
+      <c r="J5" s="23">
+        <v>15</v>
+      </c>
+      <c r="K5" s="23">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:47" s="23" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:47" s="23" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:47" s="26" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" s="26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="19"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+    </row>
+    <row r="10" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="19"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+    </row>
+    <row r="11" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="19"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+    </row>
+    <row r="12" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="19"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+    </row>
+    <row r="13" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="19"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+    </row>
+    <row r="14" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0B3638-B071-4625-AE08-F056F7C4DB64}">
+  <dimension ref="A1:AU23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="33.7109375" style="3" customWidth="1"/>
+    <col min="2" max="19" width="19.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:47" s="6" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="5"/>
+      <c r="Z1" s="5"/>
+      <c r="AA1" s="5"/>
+      <c r="AB1" s="5"/>
+      <c r="AC1" s="5"/>
+      <c r="AD1" s="5"/>
+      <c r="AE1" s="5"/>
+      <c r="AF1" s="5"/>
+      <c r="AG1" s="5"/>
+      <c r="AH1" s="5"/>
+      <c r="AI1" s="5"/>
+      <c r="AJ1" s="5"/>
+      <c r="AK1" s="5"/>
+      <c r="AL1" s="5"/>
+      <c r="AM1" s="5"/>
+      <c r="AN1" s="5"/>
+      <c r="AO1" s="5"/>
+      <c r="AP1" s="5"/>
+      <c r="AQ1" s="5"/>
+      <c r="AR1" s="5"/>
+      <c r="AS1" s="5"/>
+      <c r="AT1" s="5"/>
+      <c r="AU1" s="5"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="K2" s="11"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="K3" s="11"/>
+    </row>
+    <row r="4" spans="1:47" s="8" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="K4" s="13"/>
+    </row>
+    <row r="5" spans="1:47" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="11">
+        <v>10</v>
+      </c>
+      <c r="C5" s="11">
+        <v>20</v>
+      </c>
+      <c r="D5" s="11">
+        <v>15</v>
+      </c>
+      <c r="E5" s="11">
+        <v>15</v>
+      </c>
+      <c r="F5" s="11">
+        <v>7</v>
+      </c>
+      <c r="G5" s="11">
+        <v>5</v>
+      </c>
+      <c r="H5" s="11">
+        <v>3</v>
+      </c>
+      <c r="I5" s="11">
+        <v>15</v>
+      </c>
+      <c r="J5" s="11">
+        <v>25</v>
+      </c>
+      <c r="K5" s="11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:47" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="11">
+        <v>0</v>
+      </c>
+      <c r="C6" s="11">
+        <v>5</v>
+      </c>
+      <c r="D6" s="11">
+        <v>5</v>
+      </c>
+      <c r="E6" s="11">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11">
+        <v>2</v>
+      </c>
+      <c r="G6" s="11">
+        <v>2</v>
+      </c>
+      <c r="H6" s="11">
+        <v>2</v>
+      </c>
+      <c r="I6" s="11">
+        <v>0</v>
+      </c>
+      <c r="J6" s="11">
+        <v>5</v>
+      </c>
+      <c r="K6" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:47" s="8" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="13">
+        <v>1</v>
+      </c>
+      <c r="C7" s="13">
+        <v>0.75</v>
+      </c>
+      <c r="D7" s="13">
+        <v>0.75</v>
+      </c>
+      <c r="E7" s="13">
+        <v>1</v>
+      </c>
+      <c r="F7" s="13">
+        <v>0.6</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0.6</v>
+      </c>
+      <c r="H7" s="13">
+        <v>0.6</v>
+      </c>
+      <c r="I7" s="13">
+        <v>0.9</v>
+      </c>
+      <c r="J7" s="13">
+        <v>1.2</v>
+      </c>
+      <c r="K7" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:47" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:47" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:47" s="8" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:47" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+    </row>
+    <row r="12" spans="1:47" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+    </row>
+    <row r="13" spans="1:47" s="8" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="7">
+        <v>0</v>
+      </c>
+      <c r="C13" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="E13" s="7">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7">
+        <v>0</v>
+      </c>
+      <c r="H13" s="7">
+        <v>0</v>
+      </c>
+      <c r="I13" s="7">
+        <v>1</v>
+      </c>
+      <c r="J13" s="7">
+        <v>0</v>
+      </c>
+      <c r="K13" s="7">
+        <v>0</v>
+      </c>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+    </row>
+    <row r="14" spans="1:47" s="17" customFormat="1" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="K14" s="18"/>
+    </row>
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BADFBA24-6E42-40D7-AECA-5625F692AC5A}">
   <dimension ref="A1:AT22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -951,7 +2038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176FB67E-4120-4111-856F-436CC3C27DDB}">
   <dimension ref="A1:AT22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
(#298.2) small fix OverlapBeingDetector exclude ourself
</commit_message>
<xml_diff>
--- a/Assets/Resources/datasheets/EntitiesData.xlsx
+++ b/Assets/Resources/datasheets/EntitiesData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODING\UNITY\subrunner\Assets\Resources\datasheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A58AAA66-129A-4060-BDF4-160445C25F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090BC7B9-8BB1-4B41-BBE9-38977B63CA07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{BDB0EA0F-F215-4C7B-BC70-96EDBA517C3F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="334" xr2:uid="{BDB0EA0F-F215-4C7B-BC70-96EDBA517C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="SocialData" sheetId="6" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="56">
   <si>
     <t>Agent Type</t>
   </si>
@@ -182,28 +182,31 @@
     <t>zombo, cyber_rat, ghost, qwin</t>
   </si>
   <si>
-    <t>cat, perso, nobody, spider</t>
-  </si>
-  <si>
-    <t>rat, cat, perso, nobody, zombo, qwin</t>
-  </si>
-  <si>
-    <t>perso, zombo</t>
-  </si>
-  <si>
-    <t>rat, cat, perso, nobody, npc, spider, qwin, dev</t>
-  </si>
-  <si>
-    <t>zombo, rat, cyber_rat, perso, qwin, dev</t>
-  </si>
-  <si>
-    <t>zombo, nobody, perso, cat, spider, dev</t>
-  </si>
-  <si>
     <t>zombo, rat, cyber_rat, qwin, dev</t>
   </si>
   <si>
     <t>zombo, cat, dev</t>
+  </si>
+  <si>
+    <t>cat, bob, noby, spider</t>
+  </si>
+  <si>
+    <t>rat, cat, bob, noby, zombo, qwin</t>
+  </si>
+  <si>
+    <t>rat, cat, bob, noby, npc, spider, qwin, dev</t>
+  </si>
+  <si>
+    <t>bob, zombo</t>
+  </si>
+  <si>
+    <t>Noby</t>
+  </si>
+  <si>
+    <t>zombo, rat, cyber_rat, bob, qwin, dev</t>
+  </si>
+  <si>
+    <t>zombo, noby, bob, cat, spider, dev</t>
   </si>
 </sst>
 </file>
@@ -327,7 +330,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -375,26 +378,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -767,7 +760,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>10</v>
@@ -847,135 +840,135 @@
       <c r="I4" s="7"/>
       <c r="K4" s="13"/>
     </row>
-    <row r="5" spans="1:47" s="24" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+    <row r="5" spans="1:47" s="20" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23">
+      <c r="B5" s="19"/>
+      <c r="C5" s="19">
         <v>15</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="19">
         <v>15</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="19">
         <v>15</v>
       </c>
-      <c r="F5" s="23">
+      <c r="F5" s="19">
         <v>15</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="19">
         <v>15</v>
       </c>
-      <c r="H5" s="23">
+      <c r="H5" s="19">
         <v>15</v>
       </c>
-      <c r="I5" s="23">
+      <c r="I5" s="19">
         <v>15</v>
       </c>
-      <c r="J5" s="23">
+      <c r="J5" s="19">
         <v>15</v>
       </c>
-      <c r="K5" s="23">
+      <c r="K5" s="19">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:47" s="23" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+    <row r="6" spans="1:47" s="19" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:47" s="23" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+    <row r="7" spans="1:47" s="19" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:47" s="26" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:47" s="22" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="E8" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="26" t="s">
+      <c r="H8" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="J8" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="J8" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" s="26" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-    </row>
-    <row r="10" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-    </row>
-    <row r="11" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-    </row>
-    <row r="12" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-    </row>
-    <row r="13" spans="1:47" s="21" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="K8" s="22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
     </row>
     <row r="14" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>

</xml_diff>